<commit_message>
Auto update: 2026-01-17 17:31:16
</commit_message>
<xml_diff>
--- a/DECISION/미장_비트코인_분석.xlsx
+++ b/DECISION/미장_비트코인_분석.xlsx
@@ -613,13 +613,13 @@
         <v>23</v>
       </c>
       <c r="D4">
-        <v>95225.25</v>
+        <v>95145.28999999999</v>
       </c>
       <c r="E4">
-        <v>65.40000000000001</v>
+        <v>65</v>
       </c>
       <c r="F4">
-        <v>4.42</v>
+        <v>4.33</v>
       </c>
       <c r="G4">
         <v>60</v>

</xml_diff>